<commit_message>
module 0 and module 1.5 cleared
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/AD698-Schedule.xlsx
+++ b/data/AD698-Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\AD698-generative-ai-for-BA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25DEE542-5B75-4491-A057-2B6E3ADB697E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FB88AD2-404F-4727-8AEC-CD2267B505FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
+    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="15720" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Details" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="284">
   <si>
     <t>Assignment</t>
   </si>
@@ -875,6 +875,27 @@
   </si>
   <si>
     <t>LLM APIs (OpenAI, Gemini, Anthropic); prompt execution vs programmatic calls; API keys and secrets management; cost awareness; responsible and accountable GenAI usage.</t>
+  </si>
+  <si>
+    <t>Colab + GPU + Tensors</t>
+  </si>
+  <si>
+    <t>Compute setup, tensors, GPU execution</t>
+  </si>
+  <si>
+    <t>NN, loss, gradients, training loop</t>
+  </si>
+  <si>
+    <t>Sequence Learning Problem</t>
+  </si>
+  <si>
+    <t>Temporal modeling, intro to sequences</t>
+  </si>
+  <si>
+    <t>Agentic Systems</t>
+  </si>
+  <si>
+    <t>Math for Neural Networks, Regression and Classification Problems</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B2A5D89-D79C-44C1-8747-841FF0601386}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="4" bestFit="1" customWidth="1"/>
@@ -1682,11 +1703,11 @@
       <c r="C2" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="57" t="s">
-        <v>272</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>273</v>
+      <c r="D2" s="60" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" s="60" t="s">
+        <v>278</v>
       </c>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
@@ -1701,30 +1722,30 @@
       <c r="C3" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="D3" s="57" t="s">
-        <v>270</v>
-      </c>
-      <c r="E3" s="57" t="s">
-        <v>271</v>
+      <c r="D3" s="60" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" s="60" t="s">
+        <v>279</v>
       </c>
       <c r="F3" s="58"/>
       <c r="G3" s="58"/>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>176</v>
+        <v>274</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>216</v>
+        <v>280</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>241</v>
+        <v>281</v>
       </c>
       <c r="F4" s="58"/>
       <c r="G4" s="58"/>
@@ -1737,32 +1758,32 @@
         <v>244</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E5" s="60" t="s">
-        <v>218</v>
+        <v>241</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D6" s="60" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E6" s="60" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F6" s="58"/>
       <c r="G6" s="58"/>
@@ -1775,32 +1796,32 @@
         <v>245</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D7" s="60" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E7" s="60" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F7" s="58"/>
       <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D8" s="60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E8" s="60" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="58"/>
@@ -1813,32 +1834,32 @@
         <v>246</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D9" s="60" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F9" s="58"/>
       <c r="G9" s="58"/>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D10" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E10" s="60" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="58"/>
@@ -1851,32 +1872,32 @@
         <v>247</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D11" s="60" t="s">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="E11" s="60" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F11" s="58"/>
       <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D12" s="60" t="s">
-        <v>227</v>
+        <v>201</v>
       </c>
       <c r="E12" s="60" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="58"/>
@@ -1889,32 +1910,31 @@
         <v>248</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D13" s="60" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E13" s="60" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F13" s="58"/>
-      <c r="G13" s="58"/>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D14" s="60" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E14" s="60" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F14" s="58"/>
     </row>
@@ -1923,34 +1943,34 @@
         <v>210</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D15" s="60" t="s">
+        <v>231</v>
+      </c>
+      <c r="E15" s="60" t="s">
+        <v>232</v>
+      </c>
+      <c r="F15" s="58"/>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B16" s="60" t="s">
+        <v>282</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="D15" s="60" t="s">
+      <c r="D16" s="60" t="s">
         <v>233</v>
       </c>
-      <c r="E15" s="60" t="s">
+      <c r="E16" s="60" t="s">
         <v>234</v>
-      </c>
-      <c r="F15" s="58"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B16" s="60" t="s">
-        <v>250</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="D16" s="60" t="s">
-        <v>235</v>
-      </c>
-      <c r="E16" s="60" t="s">
-        <v>236</v>
       </c>
       <c r="F16" s="58"/>
     </row>
@@ -1959,64 +1979,39 @@
         <v>211</v>
       </c>
       <c r="B17" s="60" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D17" s="60" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E17" s="60" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F17" s="58"/>
     </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B18" s="60" t="s">
         <v>251</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D18" s="60" t="s">
-        <v>203</v>
+        <v>239</v>
       </c>
       <c r="E18" s="60" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F18" s="58"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B19" s="60" t="s">
-        <v>251</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D19" s="60" t="s">
-        <v>239</v>
-      </c>
-      <c r="E19" s="60" t="s">
-        <v>240</v>
-      </c>
       <c r="F19" s="58"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E20" s="4"/>
-      <c r="F20" s="58"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F21" s="58"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F22" s="58"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>

</xml_diff>